<commit_message>
update on march 10 morning
</commit_message>
<xml_diff>
--- a/Files/BranchList.xlsx
+++ b/Files/BranchList.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MIS\Territory Redesign\Territory\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11A5B6DB-BB7B-4848-ACE8-CD9EECB2CB1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E4C9E9-AC71-48DF-BAE8-61F98428455E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{8CC162FA-7FA8-4A68-9EC1-EACDB4AC12DC}"/>
   </bookViews>
@@ -1028,6 +1028,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8420E42-F6D0-40EB-B1CC-A10BBD4737C0}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:D203"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1051,7 +1052,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1065,7 +1066,7 @@
         <v>77.099671000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1093,7 +1094,7 @@
         <v>77.003530999999995</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>5</v>
       </c>
@@ -1107,7 +1108,7 @@
         <v>77.128750999999994</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>7</v>
       </c>
@@ -1121,7 +1122,7 @@
         <v>77.847854999999996</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>9</v>
       </c>
@@ -1135,7 +1136,7 @@
         <v>75.288602999999995</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>10</v>
       </c>
@@ -1149,7 +1150,7 @@
         <v>78.005026000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>11</v>
       </c>
@@ -1163,7 +1164,7 @@
         <v>75.109244000000004</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>12</v>
       </c>
@@ -1177,7 +1178,7 @@
         <v>79.110619</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>13</v>
       </c>
@@ -1191,7 +1192,7 @@
         <v>77.577703</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>15</v>
       </c>
@@ -1205,7 +1206,7 @@
         <v>75.057007999999996</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>18</v>
       </c>
@@ -1219,7 +1220,7 @@
         <v>75.915145999999993</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>22</v>
       </c>
@@ -1233,7 +1234,7 @@
         <v>75.569336000000007</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>24</v>
       </c>
@@ -1247,7 +1248,7 @@
         <v>78.822038000000006</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>25</v>
       </c>
@@ -1275,7 +1276,7 @@
         <v>79.380893999999998</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>27</v>
       </c>
@@ -1289,7 +1290,7 @@
         <v>77.973646000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>28</v>
       </c>
@@ -1303,7 +1304,7 @@
         <v>75.636412000000007</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>29</v>
       </c>
@@ -1317,7 +1318,7 @@
         <v>79.133382999999995</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>30</v>
       </c>
@@ -1345,7 +1346,7 @@
         <v>79.703889000000004</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>32</v>
       </c>
@@ -1359,7 +1360,7 @@
         <v>79.554565999999994</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>33</v>
       </c>
@@ -1373,7 +1374,7 @@
         <v>79.634202000000002</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>35</v>
       </c>
@@ -1387,7 +1388,7 @@
         <v>75.401307000000003</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>37</v>
       </c>
@@ -1415,7 +1416,7 @@
         <v>74.227149999999995</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>39</v>
       </c>
@@ -1429,7 +1430,7 @@
         <v>74.576626000000005</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>41</v>
       </c>
@@ -1443,7 +1444,7 @@
         <v>76.387496999999996</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>42</v>
       </c>
@@ -1457,7 +1458,7 @@
         <v>76.755435000000006</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>44</v>
       </c>
@@ -1485,7 +1486,7 @@
         <v>76.017570000000006</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>46</v>
       </c>
@@ -1499,7 +1500,7 @@
         <v>75.911186000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>47</v>
       </c>
@@ -1513,7 +1514,7 @@
         <v>78.876349000000005</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>48</v>
       </c>
@@ -1527,7 +1528,7 @@
         <v>76.534045000000006</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>49</v>
       </c>
@@ -1541,7 +1542,7 @@
         <v>77.356899999999996</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>50</v>
       </c>
@@ -1555,7 +1556,7 @@
         <v>74.530676999999997</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>53</v>
       </c>
@@ -1569,7 +1570,7 @@
         <v>74.460014999999999</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>54</v>
       </c>
@@ -1583,7 +1584,7 @@
         <v>79.284122999999994</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>56</v>
       </c>
@@ -1597,7 +1598,7 @@
         <v>77.745806000000002</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>57</v>
       </c>
@@ -1611,7 +1612,7 @@
         <v>75.015219000000002</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>58</v>
       </c>
@@ -1625,7 +1626,7 @@
         <v>77.517880000000005</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>59</v>
       </c>
@@ -1639,7 +1640,7 @@
         <v>74.009362999999993</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>60</v>
       </c>
@@ -1667,7 +1668,7 @@
         <v>77.557398000000006</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>63</v>
       </c>
@@ -1681,7 +1682,7 @@
         <v>73.860356999999993</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>67</v>
       </c>
@@ -1695,7 +1696,7 @@
         <v>74.208875000000006</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>69</v>
       </c>
@@ -1723,7 +1724,7 @@
         <v>77.015442800000002</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>71</v>
       </c>
@@ -1737,7 +1738,7 @@
         <v>74.656758999999994</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>72</v>
       </c>
@@ -1751,7 +1752,7 @@
         <v>73.935198</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>73</v>
       </c>
@@ -1765,7 +1766,7 @@
         <v>76.962166999999994</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>74</v>
       </c>
@@ -1779,7 +1780,7 @@
         <v>78.131805499999999</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>75</v>
       </c>
@@ -1793,7 +1794,7 @@
         <v>78.668348499999993</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>76</v>
       </c>
@@ -1821,7 +1822,7 @@
         <v>78.772372000000004</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>78</v>
       </c>
@@ -1835,7 +1836,7 @@
         <v>75.328823</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>79</v>
       </c>
@@ -1849,7 +1850,7 @@
         <v>78.192645999999996</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>81</v>
       </c>
@@ -1863,7 +1864,7 @@
         <v>72.537929000000005</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>84</v>
       </c>
@@ -1877,7 +1878,7 @@
         <v>76.629088999999993</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>85</v>
       </c>
@@ -1891,7 +1892,7 @@
         <v>72.967546200000001</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>92</v>
       </c>
@@ -1905,7 +1906,7 @@
         <v>73.802837999999994</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>95</v>
       </c>
@@ -1919,7 +1920,7 @@
         <v>76.125442000000007</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>96</v>
       </c>
@@ -1933,7 +1934,7 @@
         <v>76.816125999999997</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>97</v>
       </c>
@@ -1947,7 +1948,7 @@
         <v>75.668228999999997</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>98</v>
       </c>
@@ -1961,7 +1962,7 @@
         <v>80.149972000000005</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>101</v>
       </c>
@@ -1975,7 +1976,7 @@
         <v>77.016025999999997</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>102</v>
       </c>
@@ -1989,7 +1990,7 @@
         <v>79.119766999999996</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>103</v>
       </c>
@@ -2017,7 +2018,7 @@
         <v>76.565963999999994</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>105</v>
       </c>
@@ -2031,7 +2032,7 @@
         <v>76.040695999999997</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>106</v>
       </c>
@@ -2059,7 +2060,7 @@
         <v>76.342556999999999</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>108</v>
       </c>
@@ -2073,7 +2074,7 @@
         <v>76.832915</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>109</v>
       </c>
@@ -2087,7 +2088,7 @@
         <v>75.117451000000003</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>110</v>
       </c>
@@ -2115,7 +2116,7 @@
         <v>75.623388000000006</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>113</v>
       </c>
@@ -2129,7 +2130,7 @@
         <v>75.471253000000004</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>117</v>
       </c>
@@ -2143,7 +2144,7 @@
         <v>75.305484000000007</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>118</v>
       </c>
@@ -2157,7 +2158,7 @@
         <v>75.048029999999997</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>120</v>
       </c>
@@ -2171,7 +2172,7 @@
         <v>76.614040000000003</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>121</v>
       </c>
@@ -2185,7 +2186,7 @@
         <v>76.200951000000003</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>122</v>
       </c>
@@ -2199,7 +2200,7 @@
         <v>75.147644</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>124</v>
       </c>
@@ -2227,7 +2228,7 @@
         <v>76.200951000000003</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>130</v>
       </c>
@@ -2241,7 +2242,7 @@
         <v>72.953472000000005</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>132</v>
       </c>
@@ -2255,7 +2256,7 @@
         <v>70.066119999999998</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>133</v>
       </c>
@@ -2269,7 +2270,7 @@
         <v>73.017544999999998</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>140</v>
       </c>
@@ -2283,7 +2284,7 @@
         <v>70.812943000000004</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>144</v>
       </c>
@@ -2297,7 +2298,7 @@
         <v>75.796296999999996</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>145</v>
       </c>
@@ -2311,7 +2312,7 @@
         <v>74.869476000000006</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>148</v>
       </c>
@@ -2325,7 +2326,7 @@
         <v>70.786423999999997</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>149</v>
       </c>
@@ -2339,7 +2340,7 @@
         <v>72.826221000000004</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>150</v>
       </c>
@@ -2353,7 +2354,7 @@
         <v>77.833843999999999</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>151</v>
       </c>
@@ -2367,7 +2368,7 @@
         <v>79.910140999999996</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>152</v>
       </c>
@@ -2381,7 +2382,7 @@
         <v>79.984012000000007</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>153</v>
       </c>
@@ -2395,7 +2396,7 @@
         <v>77.560254</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>154</v>
       </c>
@@ -2409,7 +2410,7 @@
         <v>77.949589700000004</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>155</v>
       </c>
@@ -2423,7 +2424,7 @@
         <v>75.007632999999998</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>156</v>
       </c>
@@ -2437,7 +2438,7 @@
         <v>77.479849999999999</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>157</v>
       </c>
@@ -2465,7 +2466,7 @@
         <v>78.954155999999998</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>163</v>
       </c>
@@ -2479,7 +2480,7 @@
         <v>77.143456</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>164</v>
       </c>
@@ -2493,7 +2494,7 @@
         <v>75.702049000000002</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>165</v>
       </c>
@@ -2521,7 +2522,7 @@
         <v>76.383032999999998</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>170</v>
       </c>
@@ -2535,7 +2536,7 @@
         <v>79.732647</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>171</v>
       </c>
@@ -2549,7 +2550,7 @@
         <v>77.120808999999994</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>172</v>
       </c>
@@ -2563,7 +2564,7 @@
         <v>79.322665000000001</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>175</v>
       </c>
@@ -2577,7 +2578,7 @@
         <v>80.437470000000005</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>176</v>
       </c>
@@ -2591,7 +2592,7 @@
         <v>80.639031000000003</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>177</v>
       </c>
@@ -2605,7 +2606,7 @@
         <v>79.929286399999995</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>179</v>
       </c>
@@ -2619,7 +2620,7 @@
         <v>78.586111000000002</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>180</v>
       </c>
@@ -2633,7 +2634,7 @@
         <v>75.694051000000002</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>181</v>
       </c>
@@ -2647,7 +2648,7 @@
         <v>77.119035999999994</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>182</v>
       </c>
@@ -2661,7 +2662,7 @@
         <v>80.992503999999997</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>183</v>
       </c>
@@ -2675,7 +2676,7 @@
         <v>81.102902999999998</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>184</v>
       </c>
@@ -2689,7 +2690,7 @@
         <v>81.779065000000003</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>185</v>
       </c>
@@ -2703,7 +2704,7 @@
         <v>77.675877999999997</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>186</v>
       </c>
@@ -2717,7 +2718,7 @@
         <v>86.898128999999997</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>187</v>
       </c>
@@ -2731,7 +2732,7 @@
         <v>84.793484000000007</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>188</v>
       </c>
@@ -2745,7 +2746,7 @@
         <v>78.019333000000003</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>189</v>
       </c>
@@ -2759,7 +2760,7 @@
         <v>78.090629000000007</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>191</v>
       </c>
@@ -2773,7 +2774,7 @@
         <v>85.893152000000001</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>192</v>
       </c>
@@ -2787,7 +2788,7 @@
         <v>85.849136000000001</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>196</v>
       </c>
@@ -2801,7 +2802,7 @@
         <v>76.707447999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>197</v>
       </c>
@@ -2815,7 +2816,7 @@
         <v>81.524614</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>198</v>
       </c>
@@ -2829,7 +2830,7 @@
         <v>77.731574300000005</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>201</v>
       </c>
@@ -2843,7 +2844,7 @@
         <v>74.630962999999994</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>203</v>
       </c>
@@ -2857,7 +2858,7 @@
         <v>72.998022000000006</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>206</v>
       </c>
@@ -2871,7 +2872,7 @@
         <v>73.326058000000003</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>207</v>
       </c>
@@ -2885,7 +2886,7 @@
         <v>86.898128999999997</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>208</v>
       </c>
@@ -2899,7 +2900,7 @@
         <v>74.325638999999995</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>209</v>
       </c>
@@ -2913,7 +2914,7 @@
         <v>77.088227000000003</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>210</v>
       </c>
@@ -2927,7 +2928,7 @@
         <v>76.723613999999998</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>211</v>
       </c>
@@ -2941,7 +2942,7 @@
         <v>80.2179</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>216</v>
       </c>
@@ -2955,7 +2956,7 @@
         <v>77.305588</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>219</v>
       </c>
@@ -2969,7 +2970,7 @@
         <v>77.512570999999994</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>220</v>
       </c>
@@ -2983,7 +2984,7 @@
         <v>77.401814999999999</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>221</v>
       </c>
@@ -2997,7 +2998,7 @@
         <v>78.120912000000004</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>225</v>
       </c>
@@ -3011,7 +3012,7 @@
         <v>76.968326000000005</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>227</v>
       </c>
@@ -3053,7 +3054,7 @@
         <v>80.139885000000007</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>231</v>
       </c>
@@ -3067,7 +3068,7 @@
         <v>80.139885000000007</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>232</v>
       </c>
@@ -3081,7 +3082,7 @@
         <v>78.108027000000007</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>233</v>
       </c>
@@ -3095,7 +3096,7 @@
         <v>79.093611999999993</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148">
         <v>234</v>
       </c>
@@ -3109,7 +3110,7 @@
         <v>79.416787999999997</v>
       </c>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>235</v>
       </c>
@@ -3137,7 +3138,7 @@
         <v>82.228531000000004</v>
       </c>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151">
         <v>237</v>
       </c>
@@ -3151,7 +3152,7 @@
         <v>83.894616999999997</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152">
         <v>239</v>
       </c>
@@ -3165,7 +3166,7 @@
         <v>83.390709000000001</v>
       </c>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153">
         <v>240</v>
       </c>
@@ -3179,7 +3180,7 @@
         <v>80.045594199999996</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154">
         <v>241</v>
       </c>
@@ -3193,7 +3194,7 @@
         <v>78.507964000000001</v>
       </c>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155">
         <v>242</v>
       </c>
@@ -3207,7 +3208,7 @@
         <v>79.985485999999995</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156">
         <v>243</v>
       </c>
@@ -3221,7 +3222,7 @@
         <v>80.046442999999996</v>
       </c>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157">
         <v>244</v>
       </c>
@@ -3235,7 +3236,7 @@
         <v>78.048128000000005</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158">
         <v>246</v>
       </c>
@@ -3249,7 +3250,7 @@
         <v>78.146928000000003</v>
       </c>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159">
         <v>247</v>
       </c>
@@ -3263,7 +3264,7 @@
         <v>76.948404999999994</v>
       </c>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160">
         <v>249</v>
       </c>
@@ -3277,7 +3278,7 @@
         <v>77.296954999999997</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161">
         <v>251</v>
       </c>
@@ -3291,7 +3292,7 @@
         <v>77.504649000000001</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A162">
         <v>252</v>
       </c>
@@ -3305,7 +3306,7 @@
         <v>77.887623000000005</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A163">
         <v>254</v>
       </c>
@@ -3319,7 +3320,7 @@
         <v>78.570914999999999</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164">
         <v>256</v>
       </c>
@@ -3347,7 +3348,7 @@
         <v>78.069635000000005</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166">
         <v>258</v>
       </c>
@@ -3361,7 +3362,7 @@
         <v>80.594112999999993</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167">
         <v>259</v>
       </c>
@@ -3375,7 +3376,7 @@
         <v>77.119445999999996</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168">
         <v>261</v>
       </c>
@@ -3389,7 +3390,7 @@
         <v>78.572429650000004</v>
       </c>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169">
         <v>262</v>
       </c>
@@ -3417,7 +3418,7 @@
         <v>78.210627000000002</v>
       </c>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171">
         <v>264</v>
       </c>
@@ -3431,7 +3432,7 @@
         <v>79.895880000000005</v>
       </c>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172">
         <v>265</v>
       </c>
@@ -3445,7 +3446,7 @@
         <v>78.913394999999994</v>
       </c>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173">
         <v>266</v>
       </c>
@@ -3459,7 +3460,7 @@
         <v>79.621531000000004</v>
       </c>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174">
         <v>268</v>
       </c>
@@ -3473,7 +3474,7 @@
         <v>79.648937000000004</v>
       </c>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175">
         <v>269</v>
       </c>
@@ -3487,7 +3488,7 @@
         <v>77.703660999999997</v>
       </c>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176">
         <v>270</v>
       </c>
@@ -3501,7 +3502,7 @@
         <v>77.784942000000001</v>
       </c>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177">
         <v>271</v>
       </c>
@@ -3515,7 +3516,7 @@
         <v>77.540797999999995</v>
       </c>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178">
         <v>272</v>
       </c>
@@ -3543,7 +3544,7 @@
         <v>78.034673999999995</v>
       </c>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180">
         <v>274</v>
       </c>
@@ -3557,7 +3558,7 @@
         <v>78.484643000000005</v>
       </c>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181">
         <v>276</v>
       </c>
@@ -3571,7 +3572,7 @@
         <v>78.427306999999999</v>
       </c>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182">
         <v>277</v>
       </c>
@@ -3599,7 +3600,7 @@
         <v>78.155985000000001</v>
       </c>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184">
         <v>279</v>
       </c>
@@ -3613,7 +3614,7 @@
         <v>77.299143000000001</v>
       </c>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185">
         <v>280</v>
       </c>
@@ -3627,7 +3628,7 @@
         <v>77.379606999999993</v>
       </c>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186">
         <v>281</v>
       </c>
@@ -3655,7 +3656,7 @@
         <v>77.871754999999993</v>
       </c>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188">
         <v>283</v>
       </c>
@@ -3669,7 +3670,7 @@
         <v>78.058168100000003</v>
       </c>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189">
         <v>285</v>
       </c>
@@ -3683,7 +3684,7 @@
         <v>82.547014000000004</v>
       </c>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190">
         <v>288</v>
       </c>
@@ -3697,7 +3698,7 @@
         <v>82.000373999999994</v>
       </c>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191">
         <v>289</v>
       </c>
@@ -3711,7 +3712,7 @@
         <v>81.725345000000004</v>
       </c>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192">
         <v>290</v>
       </c>
@@ -3725,7 +3726,7 @@
         <v>80.290156999999994</v>
       </c>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193">
         <v>291</v>
       </c>
@@ -3739,7 +3740,7 @@
         <v>81.135957000000005</v>
       </c>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194">
         <v>292</v>
       </c>
@@ -3753,7 +3754,7 @@
         <v>77.219300000000004</v>
       </c>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195">
         <v>293</v>
       </c>
@@ -3767,7 +3768,7 @@
         <v>77.452563999999995</v>
       </c>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A196">
         <v>296</v>
       </c>
@@ -3781,7 +3782,7 @@
         <v>76.938862200000003</v>
       </c>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197">
         <v>298</v>
       </c>
@@ -3795,7 +3796,7 @@
         <v>77.972453000000002</v>
       </c>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A198">
         <v>299</v>
       </c>
@@ -3809,7 +3810,7 @@
         <v>77.214580999999995</v>
       </c>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199">
         <v>302</v>
       </c>
@@ -3823,7 +3824,7 @@
         <v>76.613290000000006</v>
       </c>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200">
         <v>333</v>
       </c>
@@ -3837,7 +3838,7 @@
         <v>77.241975920000002</v>
       </c>
     </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201">
         <v>353</v>
       </c>
@@ -3851,7 +3852,7 @@
         <v>77.136281999999994</v>
       </c>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202">
         <v>356</v>
       </c>
@@ -3865,7 +3866,7 @@
         <v>77.274699999999996</v>
       </c>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203">
         <v>378</v>
       </c>
@@ -3880,7 +3881,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D203" xr:uid="{B8420E42-F6D0-40EB-B1CC-A10BBD4737C0}"/>
+  <autoFilter ref="A1:D203" xr:uid="{B8420E42-F6D0-40EB-B1CC-A10BBD4737C0}">
+    <filterColumn colId="1">
+      <customFilters>
+        <customFilter val="k*"/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>